<commit_message>
added all human reviews
</commit_message>
<xml_diff>
--- a/qualitative_evaluation/all_human_reviews.xlsx
+++ b/qualitative_evaluation/all_human_reviews.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eveyhuang/Documents/NICO/ai-scientist/qualitative_evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{518AD3D3-7327-D14B-82F4-768AF2705A58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B144B5E-9B06-4245-890E-C63930B72B27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="23840" yWindow="7640" windowWidth="28040" windowHeight="17440" xr2:uid="{63BAB5CA-8E1E-9346-9166-AF00D28F74E3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="262">
   <si>
     <t>year</t>
   </si>
@@ -229,12 +229,768 @@
   <si>
     <t>The project aims to identify genes differentially  expressed between plant species that exhibit cytokinetic arrest  during heat stress and those that don't from 12 publicly available  single-cell transcriptomics data. Specifically, lists of genes co expressed with known cytokinesis genes will be generated for each  plant species and compared to identify genes or alleles that change  upon heat stress. The motivation for the work is important as heat  stress threatens plant yields and food security. However, the  proposal left unclear whether 12 datasets from multiple species  and experimental conditions would be sufficient to narrow the  number of genes to be tested following the bioinformatics analysis- -given how complex single-cell data is, such an estimate would have  made the project less risky. Furthermore, preliminary data in the  proposal did not single out noteworthy genes that could help  validate the bioinformatics analysis results, and the proposal left  unclear what tests (and throughput) would be used to validate the  predictions of the bioinformatics analysis.</t>
   </si>
+  <si>
+    <t>Elucidating genome structure-function relationships in human brain cells</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Justification:This project specifically focuses on the comprehensive genomic framework of the brian cell, aiming to understand the cell-type-specific gene expression at the single cell level. The group also focuses on the datasets relevant to AD patients, with a great potential for neuro-degerative diseases. 
+Multiple machine learning and generative models will be proposed or used in the project. multiple group members are experts in the respective fields of genome biology, bioinformatics, AI, and neural degenerative diseases. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multiple established AI models could be directly leveraged. Given the team's strong expertise in AI and single cell based applications, there is strong confidence that the project will be implemented in a good pace.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The datasets are well-defined from the work group's prior publications or other public available datasets. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generative models will be shared, and the processed data will be shared as well. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Great team work proposing innovative approaches to address fundamental questions in genome biology, while leading to signficant clinical and scientific impacts. </t>
+  </si>
+  <si>
+    <t>There is a need for new tools to integrate different types of single-cell genomics data to provide new insights on the link between chromatin organization and gene expression. I do not have the expertise to comment on the rigor of the modeling approach. However, the PIs propose training these models using a very limited number of datasets (which they acknowledge). It is unclear if the project is feasible given the number of available datasets</t>
+  </si>
+  <si>
+    <t>The timeline seems reasonable, given ther requested resources.</t>
+  </si>
+  <si>
+    <t>The project synthesizes multiple single-cell datasets, however the total number of datasets is limited. The PIs provide a table of all datasets to be used, but not all are discussed in the proposal text. Not clear where dataset 6 fits in.</t>
+  </si>
+  <si>
+    <t>There was no discussion of a commitement to open, reproducible science.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With single-cell sequencing rapidly expanding in scope, new models to integrate data are needed to link genome structure and gene expression. The proposal integrates a strong working group to develop new models to analyze these datasets. The main weakness with the proposal is it is unclear whether the limited number of available datasets are sufficient to train the models and achieve the proposed goals. It is also unclear how all the datasets fit into the proposal. The proposal could also be strengthened by demonstrating a clear commitment to open science. </t>
+  </si>
+  <si>
+    <t>1. linking 3D chromatin organization (a mesoscale structure) to gene expression and cellular diversity is important 
+2. using AI-based multimodal integration to tackle long-standing challenges in understanding genome architecture is innovative 
+3. it is not clear how the team will compare their finding with existing models/tools
+4. reliance on pretraining non-brain datasets introduces potential risks that require additional mitigation strategies</t>
+  </si>
+  <si>
+    <t>1. The timeline is ambitious, especially given the computational and experimental challenges 
+2. The lack of co-assay data for brain cells may introduce delays
+3.Risk management plans could be expanded to strengthen feasibility</t>
+  </si>
+  <si>
+    <t>1. Integration of multiple data modalities and disciplines (neurobiology, genomics, AI) 
+2. Data sources are clearly described with limitation properly acknowledged. However, strategies for handling missing or incomplete datasets could be more detailed.</t>
+  </si>
+  <si>
+    <t>Explicit sharing of tools and datasets is included, though more detail on dissemination strategies would further strengthen this commitment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The proposal aims to use generative AI to integrate multimodal single-cell genomic data, uncovering how 3D chromatin organization drives gene expression, neuronal diversity, and epigenetic changes in Alzheimer’s disease. It introduces two tools: scCOE for analyzing structural variation and scGEP for predicting gene expression from chromatin architecture. By leveraging advanced AI techniques like transformer models and contrastive learning, the project seeks to understand genome structure-function relationships and neurodegeneration.
+The key strengths includes (1) strong focus on addressing mesoscale emergent phenomena in genome organization, (2)
+Innovative and interdisciplinary approaches with potential for impactful advancements, (3) Well-qualified team with complementary expertise, and (4) Commitment to reproducibility and open science principles. Key areas for improvement includes (1) Ambitious timeline with limited contingency planning for delays, and (2) Transferability of pretraining non-brain datasets could pose risks. </t>
+  </si>
+  <si>
+    <t>MaiTool - LLM-powered bioinformatics tools for microbiome analysis</t>
+  </si>
+  <si>
+    <t>Relevance to Emergent Phenomena: The project integrates large language models (LLMs) with bioinformatics tools, enabling AI-assisted microbiome research. While it does not directly address emergent mesoscale biological phenomena, it supports interdisciplinary synthesis of microbiome datasets.
+•	Novelty &amp; Significance: The proposal is highly innovative, bridging natural language processing (NLP) and bioinformatics. By integrating LLMs with bioinformatics workflows, MaiTool has the potential to revolutionize microbiome data analysis.
+•	Rigor of Approach: The methodology is well-defined, involving LLM fine-tuning, API development, and bioinformatics pipeline integration. However, additional details on how LLM outputs will be validated against existing bioinformatics tools would strengthen the proposal.
+Justification: The project is highly novel and well-structured but could further clarify its contribution to mesoscale biological phenomena and its validation strategies for LLM-assisted analysis</t>
+  </si>
+  <si>
+    <t>•Scope &amp; Timeline: The project proposes a two-year timeline with clear milestones, including LLM evaluation, API development, and software deployment.
+•Potential Challenges: Training and fine-tuning LLMs for specialized microbiome queries could present computational and data limitations. The proposal should discuss how false positives/negatives from LLM-assisted queries will be minimized.
+Justification: The scope and timeline are realistic, but validation of AI-assisted bioinformatics workflows needs further discussion.
+Justification: The scope and timeline are realistic, but validation of AI-assisted bioinformatics workflows needs further discussion.</t>
+  </si>
+  <si>
+    <t>•Synthesis Focus: The project aligns well with NCEMS’s data synthesis mission, focusing on integrating and reanalyzing existing microbiome datasets rather than generating new data.
+•Data Identification: The proposal provides a detailed data source inventory, including MGnify, MG-RAST, HMP, IMG/M, SRA, and others. It also discusses API development for seamless data integration.
+Justification: The proposal demonstrates a strong understanding of available microbiome data sources and their limitations.</t>
+  </si>
+  <si>
+    <t>Commitment to Open Science: The proposal emphasizes open-source tool development (MaiTool), dataset integration, and API access. The team commits to making datasets and code publicly available on GitHub.
+Justification: The project aligns well with NCEMS’s open science principles.</t>
+  </si>
+  <si>
+    <t>The MaiTool proposal presents an innovative, interdisciplinary approach to integrating LLMs with bioinformatics tools for microbiome analysis. The project aligns well with NCEMS’s mission, leveraging existing microbiome datasets, AI-driven insights, and open-access bioinformatics workflows.
+Minor refinements could strengthen the proposal, particularly regarding validation of AI-assisted analyses, cost-efficiency of LLM fine-tuning, and mitigation of false positives in automated queries. Overall, the project has high potential for impact and is strongly recommended for funding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strength: 
+The study of microbiota is inherently related to emergent phenomena in complex systems. The tool, if developed would be very useful and novel. 
+Weakness:
+The application is quite vague on what MaiTool will be able to do and how the team will go about developing MaiTool. They end up focusing on details like the REST API when much more important factors such as how the model would be trained, what it would be trained to do, etc... are missing. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The scope is not clear. In fact, the first step of the project seems to be to figure out the scope. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">There is a clear synthesis aspect to the project and the authors have identified many large data sources that would be appropriate. </t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>The applications vision is significant and novel. What is lacking is scope, expertise, and methodologic details</t>
+  </si>
+  <si>
+    <t>This proposal aims to develop MaiTool as an interface for retrieving microbe-related data from publicly accessible libraries and for performing "lightweight analyses". It is not clear what kind of analyses the tool will perform and how this tool stands out from other current interfaces. In the example given, it is not clear what patterns and relationships involving the test organism the tool will explore—this is important to understand the tool's applicability.</t>
+  </si>
+  <si>
+    <t>While I'm not an expert on the timeline for a bioinformatics tool and LLM development project and the potential pitfalls that may arise, the outlined timeline is clear and detailed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> This tool appears to be a layer above the current GPT models with additional quality control. The team proposes that this tool will perform visualization and statistical analysis for retrieved data. The data sources were identified but no limitations were acknowledged.</t>
+  </si>
+  <si>
+    <t>The proposal demonstrates commitment to open science principles</t>
+  </si>
+  <si>
+    <t>This is a good proposal for developing  MaiTool as an interface for retrieving microbe-related data from publicly accessible libraries and performing some analyses. The tool will prioritize quality data better than existing GPT models, and the working group is comprised of experts who will contribute to the success of the project. However, it is unclear what kind of analyses the tool will provide and the applicability of the tool to the broader community.  </t>
+  </si>
+  <si>
+    <t>The proposal would like to combine the LLM tool with bioinformatics tools for microbiome analysis, which could kind of improve the current LLM capabilities in microbiome field, but not to address emergent phenomena, also not that innovative.</t>
+  </si>
+  <si>
+    <t>I do not have expertise in bioinformatics, and can not give an objective justification.</t>
+  </si>
+  <si>
+    <t>The proposal clearly demonstrates a synthesis project and the data sources are explicitly identified, but do not acknowledge the limitations.</t>
+  </si>
+  <si>
+    <t>Yes, the proposal does</t>
+  </si>
+  <si>
+    <t>The proposal would combine LLM and bioinformatics tools to develop a model for microbiome analysis as well as ancient DNA research. The team consists of professors with diverse backgrounds in bioinformatics, ancient microbiomes and data modelling. The proposal is kind of a plain combination, it could improve the current LLM capabilities for visualizing dataset profiles but is short of strength and doesn't address emergent phenomena because it stays on visualizing dataset profiles.
+Since microbiomes are closely related to environment, disease and food safety, is it possible to develop a LLM-powered cutting edge tool to provide insightful information on environmental protection, disease prevention, drug and antibiotic development? It would significantly empower researchers.</t>
+  </si>
+  <si>
+    <t>Synthesizing gene expression data to create an atlas of bacterial cell states</t>
+  </si>
+  <si>
+    <t>The researchers propose to investigate an exciting and important phenomenon - linking gene expression data to cell states has groundbreaking potential for our understanding and application of microbial physiology. The rationale is well-grounded and a robust approach is presented through merging datasets from many different sources and methods (microarrays and RNA-seq). The project builds from merging and integrating data to analzying, testing, and building a predictive classifier, and includes preliminary analysis with the existing Monocle 3 algorithm</t>
+  </si>
+  <si>
+    <t>The project is well thought out and clearly outlined, though it seems quite ambitious; the timeline is logically laid out, but I am unsure all of the proposed tasks can be accomplished in the given time frame. The proposal did not address potential roadblocks that may impede progress and/or how they will be navigated.</t>
+  </si>
+  <si>
+    <t>Data sources are clearly identified via NCBI SRA and GEO databases as well as existing E. coli databases. Selection of data for non-E. coli species is a little less clear (a few example species are listed, but not all are planned out). Limitation due to lack of metadata is acknowledged, but the impact is not fully addressed</t>
+  </si>
+  <si>
+    <t>Open science is addressed with concrete actions (open-source code and datasets, licensure, documentation, etc.) and includes a plan for advertisement and dissemination.</t>
+  </si>
+  <si>
+    <t>The researchers propose an exciting and innovative idea with strong benefit for the scientific community, providing useful and potentially transformative output. The project is ambitious with a tight timeline, spanning data integration, analysis, and construction of a cell state classifier. The project is truly a synthesis project, with the potential to produce emergent knowledge. In further developing the project, the goal of applying the classifier to microbial communities is currently vague, and the link to evolution (as mentioned in the abstract and in Hypothesis 3), while conceptually interesting and important, feels only weakly connected in the current description.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Although the proposal does not explicitly bridges scales, as it stays in the gene expression realm, it does deal with the emergent property of cellular states. These cellular states are broadly defined and the proposal looks at a way to describe and unveil more states by synthetizing existing data sets.
+Even though the novelty is not necessarily on the methodology, its relevance is in addressing a need to have a uniform analysis and much needed quality control for large amounts of expression data available from multiple sources.
+The proposal is well motivated, clearly delineated and methodologies, hypothesis and expected outcomes well presented. </t>
+  </si>
+  <si>
+    <t>The data processing, quality control and analysis goals for both E. coli and "Other organisms" data sets seem feasible and well planned. It was less clear to me, how the final pipeline will be used by the scientific community. The proposal mentions sharing software containers and having them maintained by the community. Do they mean that documentation, tutorials and code will not be done by the working groups in this proposal? It was unclear to me.</t>
+  </si>
+  <si>
+    <t>This is one strenght of this proposal, it is clearly a synthesis project that is much needed and might help accelerate further discovery. Current fragmentation of gene expression data is an issue and a uniform way to process, clean and visualize a large body of data is needed. Data sources are clearly listed and no limitations have been made explicit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The proposal does a great job justifying and providing support for open and reproducible science principles, making it one of the strenghts of this proposal. The need for a community based resource that integrates and process important gene expression data in a unified way is highlighted. The proposal also describes the importance of generating clear documentation, tutorials and easy to use softaware pipelines. Less clear to me would be the fate of the project past 2 years of development. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strengths of this proposal include the identification of a clear need to synthesize gene expression data into cellular states that fit well into the NCEMS goal of finding emergent properties from multiple sources of data. The plan is clearly structured and the unification, quality control and ML plans for data analysis and visualization seem significant. The proposal highlights principles of reproducible data and motivates well the plan objectives with those principles. The group has the expertise and knowhow to accomplish the goals.  Some areas for improvement include a proper determination of how NCEMS resources could boost the success of the grant. More details on how the pipelines will be used by the community other than mentioning software containers. How will the plan mitigate the issue of maintainace after 2 years. Finally, the use of UMAP has been lately critisized by some members of the scientific community, therefore providing more alternatives for more modern ML technologies migth help improve the proposal.  </t>
+  </si>
+  <si>
+    <t>The connection of gene expression data to cell state in E. coli addresses the mesoscale and how gene expression leads to the emergent phenomena of cellular state. 
+Novely comes primarly from the quantity of data that will be combined, as well as the integration of microarray and RNA-seq datasets. There are some intermediate projects (for example normalized RNA-seq gene expression by read length, combinining microarray and RNA-seq) that are interesting in and of themselves.
+The methodology and approach are described at high-level, perhaps in part due to the limited space. At a high level, in general the approach seems logical. However, some details such as how data harmonization will be done and verified, are not described in a way at they can be carefull assessed</t>
+  </si>
+  <si>
+    <t>The timeline and scope are realistic within a two year timeframe. Perhaps it would make sense to start developing the classifier earlier for E. coli data alone. Synthetic data could be used to check that the classifier works for mixed E. coli datasets. There is limited discussion of alternative approaches. For example, presumably if the RNA-seq and microarray data cannot be integrated, the project can move forward, but these routes are not delineated.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is a synthesis focused project which will leverage existing E. coli gene expression data sets to create an atlas of cell states. The data sources are identified, and some limitations such as poor metadata, are discussed. The datasets and quantity of data that will be combined is exciting. </t>
+  </si>
+  <si>
+    <t>The proposal does mention wanting to follow FAIR principles. However, specific resources, including how data will be distributed and how software will be made reusable are not specified. It is mentioned that this is an area where they would like to engage CMERCs expertise to ensure adherence to best practices for open science.</t>
+  </si>
+  <si>
+    <t>The overarching goal of this proposal is to combine existing E. coli and other bacterial bulk gene expression data to create an atlas of bacterial cell states and then use this framework to create a classifier that predicts cell state composition in populations of bacterial cell using metatranscriptomic data. This will be completed in three primary activities (1) developing the ingest pipeline to harmonize bacterial gene expression data from microarray and RNA-seq, (2) using dimensional reduction to identify cell states, or attractors in the reduced space and (3) generating a classifier to predict cell state distributions in populations. Three software/data products will be produced (1) inGEST, (2) an atlas of cell states with visualization tools and (3) a classifer that will take bacterial gene expression dataset and predict cell state composition (including data from communities with multiple species) . Strengths of the proposal include the amount of data that will be synthesized in order to generate the most comprehensive understanding of E. coli (and potentially other bacterial species) cell state to date. Colllaboration with CMERC is appropriate, though sometimes minimally described, particularly if it will make the infrastructure developed in this proposal more likely to be distributed, and reusable. I think that the focus on E. coli and bacteria is particularly exciting, particularly given the lack of utility of current scRNA-seq approaches in this space. The ability to delineate cell populations from bulk data would be transformational.
+The proposal would be strengthend by consideration of alternative approaches, more details of how their results would be validated, and a closer integration with CMERC. Some important details of the approach are missing, for example how the classifer can be extended to multiple species and how the data harmonization will be done</t>
+  </si>
+  <si>
+    <t>Relevance to Emergent Phenomena: The proposal aims to synthesize bacterial gene expression data using machine learning, which aligns well with emergent mesoscale phenomena in molecular and cellular biosciences. The project seeks to identify fundamental bacterial cell states and transitions, which are key to understanding microbial behavior and adaptation.
+•	Novelty &amp; Significance: The approach is innovative, integrating large-scale transcriptomics data with machine learning to construct a Bacterial Cell State Atlas. If successful, this will provide an unprecedented resource for understanding bacterial physiology and evolution.
+•	Rigor of Approach: The methodology is robust, leveraging existing datasets and incorporating dimensional reduction, orthologous gene mapping, and machine learning classifiers. However, the proposal would benefit from more details on how variability across datasets will be handled.
+Justification: The project presents a novel and well-structured approach to bacterial gene expression synthesis and classification, with strong potential to advance the field.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Scope &amp; Timeline: The project’s two-year timeline is reasonable, with a logical progression from E. coli datasets to broader bacterial species.
+•	Potential Challenges: Integrating heterogeneous datasets from different experimental conditions may introduce noise that could affect classifier performance. The proposal would benefit from more discussion on data harmonization strategies.
+Justification: The project is well-scoped and feasible, but challenges in data harmonization and classifier validation should be addressed in greater detail</t>
+  </si>
+  <si>
+    <t>Synthesis Focus: The proposal clearly aligns with NCEMS's mission of synthesizing existing data rather than generating new experimental data.
+•	Data Identification: The team provides a comprehensive dataset inventory, including GEO, SRA, and curated bacterial expression databases such as OKgeneExpDB and PRECISE-1K. They acknowledge data quality concerns and propose strategies for standardization.
+Justification: The proposal demonstrates a strong understanding of existing data sources and synthesis methods.</t>
+  </si>
+  <si>
+    <t>Commitment to Open Science: The project commits to open-access principles, including the development of open-source tools (InGEST pipeline), dataset sharing, and GitHub-based collaborative maintenance.
+Justification: The proposal strongly aligns with NCEMS’s open science mission</t>
+  </si>
+  <si>
+    <t>Narrative Summary:
+This proposal presents an innovative and well-structured approach to synthesizing bacterial gene expression data into a Bacterial Cell State Atlas. The project has high scientific merit, strong feasibility, and a well-qualified interdisciplinary team. The proposed work aligns well with NCEMS’s mission of data synthesis and open science.
+Minor refinements could strengthen the proposal, including more details on data harmonization strategies and alternative computational efficiency approaches. Nonetheless, the project has high potential for impact and is strongly recommended for funding.</t>
+  </si>
+  <si>
+    <t>Energetic Origins of Connectivity within Protein Interaction Networks</t>
+  </si>
+  <si>
+    <t>IDRs have long been thought to be protein-protein interaction hubs, and so the proposal that this can be quantified in terms of network organization doesn't seem particular innovative.   The focus on marginally stable proteins is perhaps more innovative, but the knoweldge gap is still not clearly articulated.</t>
+  </si>
+  <si>
+    <t>The details in the proposal are not sufficient for determining feasibility. There are still large knowledge gaps, e.g. about how mutations affect IDP-binding interactions that were not carefully considered</t>
+  </si>
+  <si>
+    <t>It would seem that fairly simple analysis of existing network models (e.g. pulling out the disordered proteins) can get at some of the underlying questions.  I wasn't clear on why so many computational resources would be required</t>
+  </si>
+  <si>
+    <t>Not particular discussed, so not clear.</t>
+  </si>
+  <si>
+    <t>The proposal aims to determine how unstable or intrinsically disordered proteins interface with protein-protein network topology.  The role of chaperones as secondary points of connectivity, as well as of the unique role in these proteins types in their promiscuity are all interesting questions. 
+However, the details and connections between the aims lead to some concerns about the approach.  For example, proteins of marginal stability, according to the text, can be made more or less stable with single point mutations, but structure prediction is often relatively insensitive to mutation.  The overall argument feels a bit circular, that is IDPs that are more promiscusous are expected to be more promiscuous.  How do the authors propose to determine which IDRs are more promiscucous, other than the degree of connectededness in the networks, arising from (I presume) protein-protein interaction databases.  The evolutionary models given for folded proteins aren't clearly adaptable to intrinsically disordered proteins, or at least absent models of binding interactions, I'm not sure how to quantify mutational affects on binding affinity.  Moreover, proteins tend to be organized into domains, with few proteins being fully disordered or fully ordered.  It's unclear if the authors have considered even how to define a disordered protein, and that the degree of disorder may be variable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The proposal aims to use the knowledge on intrinsically disordered proteins (IDP) and extend it to the proteins that do not manage to fold correctly in vivo (defined as “intrinsically unstable” forms – which the abstract states represent 10% of all proteins - citation?). The investigators propose to use network analysis AI assisted tools and various databases of protein stability and genes. The main hypothesis is that IDPs  play an important role in network communication while in their unstructured form, which drives the need of the investigators to make a connection between IDPs and intrinsically unstable forms of otherwise structured proteins. The major weakness of this proposal seems to come from the difficulty to assess for a given protein how much of the expressed molecules are intrinsically unstable. In the database table, I could only find one reference to assess protein stability - ProThem (source ID 7) – which also does not seem to provide the needed information. However, assuming that the PIs identify a folding/stability free energy database (which is also used as input in the P_native formula), it is not clear how the thermal stability of proteins measured in vitro, in the absence of any chaperones, can be related to propensity of a protein to be in an “intrinsically unstable” form in vivo, where chaperones help with folding. </t>
+  </si>
+  <si>
+    <t>Timeline is appropriate. However, the provided technical details are insufficient. For example, it is not clear how evolutionary models will be fine-tuned. More specific, from the definition of P_native, if a protein and chaperone do not interact (gamma=0), the formula produces a value of 0.5, which seems incorrect to me, and I could not find in the references cited an explanation on this. Does this mean on average, in the absence of chaperones, proteins have 0.5 probability to fold in their native form?
+AI based models will have the natural tendency to predict the stable structures as they are occurring with higher probability, and it is not clear how the PIs intend to bias them for the  “intrinsically unstable” forms. How will they even be trained, given that there are no structure of the unstable forms? Is there a way to assess these predictions experimentally? Maybe knocking-out a protein from a “party hub”?</t>
+  </si>
+  <si>
+    <t>The proposal justifies the synthesis focus. However, some libararies do not seem to be correctly referenced and there is limited discussion on the shortcomings of the selected data bases</t>
+  </si>
+  <si>
+    <t>The proposal does not seem to address this point.</t>
+  </si>
+  <si>
+    <t>Trying to connect protein instability with their role in the interaction network is an interesting idea. However, there are some concerns on the currently available information to accomlish this task.</t>
+  </si>
+  <si>
+    <t>This proposal deals with an important question connecting cellular scales (protein interaction networks) with molecular aspects of protein stability and folding. 
+Although methods per se are not particularly innovative, as a whole they aim to solve an innovative question for which there is no answer yet. 
+Methodology is clearly explained and the three goals are logically connected in the form of network acquisition, network biophysical characterization and network evolution (simulation).</t>
+  </si>
+  <si>
+    <t>Given the prior work by the groups involved and the description of the research, the time frame and amount of work seems completely feasible for 4 expert labs. My only concern would be if the results will actually identify a causal relationship between protein stability and network topology. Given the complexity of biological networks, I would be skeptical the topology would be fully explained by this biophysical properties that are typically fine tuned by individual selection processes.</t>
+  </si>
+  <si>
+    <t>Data sources are clearly delineated and listed involving interaction networks, ontology data, LiPMS and expression datasets. No limitations were discussed about the data per se, the authors centered in this being a new direction of their group therefore requiring support to pursue it.</t>
+  </si>
+  <si>
+    <t>I could not find a explicit statement related to reproducible science principles, there is no evidence that suggests that the outcomes of this proposal will be closed to the scientific community. A statement of software outcomes and their plans to make them accessible would have been ideal.</t>
+  </si>
+  <si>
+    <t>This proposal fits well within the goals or data re-use and the idea of bridging biological scales. The goal of providing biophysical/molecular explanatinons to network phenomena and properties at the cellular scale is relevant. Another strength is the expertise of the groups and the connectivity between the proposal goals and the scientific methodologies. 
+Some areas of improvement include providing evidence that there might be a real causal relationship between stability and a large scale phonomenon like scale-free networks. A better justification is needed of the requirement of staff to help with data curation and a more explicit statement about how the results will be available for reproducibility and open science.</t>
+  </si>
+  <si>
+    <t>The project clearly addresses an emergent phenomenon (PPI network scaling), and connects this to interesting questions in evolution and biophyscs
+* While others have compared PPI network structure across species, the authors open new and interesting hypotheses about the role of chaperones, unstable proteins and IDPs in setting network architecture.
+* In general the approach was clear, however the methodology behind the simulations in goal 3 was harder to follow (what do GA "steps" look like and what is the objective function? I am thinking the networks are maybe (reduced size?) toy networks, or will you start with a natural network for simulation? how will you evaluate network degeneracy and compare architecture between simulated and natural networks?) - some of this may be due to limited space to describe a complex simulation.</t>
+  </si>
+  <si>
+    <t>The proposed division of labor amongst the groups is clear, and the milestones are reasonable. It would be useful to have approximate times attached to each milestone under the time line.</t>
+  </si>
+  <si>
+    <t>The project clearly makes use of extant data to begin addressing an emergent property of molecular systems. I can see the reconstructed PPI networks and associated annotations having broad utility beyond this working group. I did not see where they would get the data for the C. elegans PPI network reconstruction, but am presuming it exists. It was also not clear where they will get annotations for chaperones or oligomers in each organism (milestone 4)</t>
+  </si>
+  <si>
+    <t>The proposal is well structured for team science, however I did not see an explicit discussion of open or reproducible science principles.</t>
+  </si>
+  <si>
+    <t>This proposal brings together expertise in omics, evolution, systems biology, and biophysics to understand how IDPs and protein stability influence network architecture. The overall biological question is interesting, and the work has potential to yield new resources (curated PPI networks with annotations) that are useful beyond the scope of this proposal. While the methodology for goals 1 and 2 felt reasonably clear, the evolutionary simulations and process for evaluating outcomes in goal 3 was more difficult to understand. That said, I like the idea of blending simulations with analysis of extant data - this is a nice combination.</t>
+  </si>
+  <si>
+    <t>Elucidating emergent structures in cellular RNA-protein interaction networks</t>
+  </si>
+  <si>
+    <t>The proposal certainly addresses emergent phenomena at the mesoscale and addresses questions of significant importance in RNA biology and gene regulation. However, there are few weaknesses or parts of confusion thus dimish the clarity: (1) Throughout the proposal, the investigators mention that they aim to build a predictive framework, but it's often unclear what exactly they are aiming to predict. More importantly, it's unclear throughout the proposal which statistical model they are proposing to use to develop a prective model and how they will account for the variable background (signal to noise) issues across disparate datasets and datatypes.</t>
+  </si>
+  <si>
+    <t>The timeline and scope of the project seems overly ambitious given the extent of data types that the investigators are hoping to integrate over and analyze.</t>
+  </si>
+  <si>
+    <t>Data sources are explicitly identified and encompass a diverse set of techniques, biological scales, and types of molecules being assayed. The investigators have done a nice job identifying a comprehensive set of data from the same cell type, making the biology more streamlined. The proposal is clearly a synthesis project across different scales of RNA biology. However, there is less information about the limitations of the data sources and data types - most of the analysis questions are focused on integrating datasets to create databases or maps of interactions, but less mention is made about how to clean up datasets to avoid missing data problems or correct for biases between data types that might influence the probability of observing interactions</t>
+  </si>
+  <si>
+    <t>Team talks about creating open-source tools and making biological databases and "maps" generated by their analyses publically available. It would be great to also ensure that all intermediate code was also made publically available to enable these types of meta-analyses in the future.</t>
+  </si>
+  <si>
+    <t>This is a generally well-written and well-rationalized proposal from a strong and diverse team of investigators. They propose to integratively analyze sequencing, proteomic, imaging, and other datatypes that inform about mRNA-protein and RNA-binding protein interactions. The proposal address an important knowledge gap in RNA biology and certainly revolves around shedding light around an emergent phenomena at the mesoscale. My major worries are that their proposal is a bit too ambitious in it's scope, with the aim to integrate across too many datasets and build too many predictive models (the statistical basis of which is hard and not sufficiently described in the proposal) in a two year timeframe. It would be useful to have a more precise set of biological questions and perhaps even hypotheses laid out that can be addressed with these analyses.</t>
+  </si>
+  <si>
+    <t>Predicting RNP composition by merging data from diverse and disparate assays is an innovative approach which will allow identification of emergent behaviour of different proteins and RNA coalescing to perform unique functions at the mesoscale. Results from this study will expand our knowledge of RNA and protein interactions in context of possible cumulative and combinatorial function and provide insights about possible effects of genetic or environmental perturbations. The use of linked features for integrating disparate datasets is a bit unclear, and might be explained better with an example.</t>
+  </si>
+  <si>
+    <t>Given the number of researchers expected to be involved in participating research groups, and the support of NCEMS, the goals and milestones are feasible.</t>
+  </si>
+  <si>
+    <t>Proposal involves integration of existing data, requires diverse and distinct areas of expertise which is provided by the three participating labs, and will provide novel insights about RNP structure and function. Datasources have been explicitly identified. Limitations of datasets individually and after integration have not been adequately explained.</t>
+  </si>
+  <si>
+    <t>Team commits to release the findings of proposal in form of an open access tool and open access publications.</t>
+  </si>
+  <si>
+    <t>Team proposes an innovative approach to characterize and predict the composition  of RNPs, and predict its effect on emergent function of RNPs under perturbed conditions by integrating disparate publicly available datasets. Successful execution of this project will provide useful insights in the fields of RNA biology, and emergent biological propoerties in general. The participating labs have the necessary expertise to execute this project successfully. This proposal satisfies the conditions of a synthesis project and the team has adequtely demonstrated its need for NCEMS support. 
+It could have made the proposal stronger if the team delved into the specifics of integrating disparate datasets using linked features and also explain strategies for normalizing and integrating metrics from such disparate datasets, and highlight an example. While the team has provided strategies for validating their predictions and models, the proposal could have further improved if the team described potential caveats of individual dataset types that they propose to integrate, and how much of these caveats would still remain after integrating the datasets have been integrated.</t>
+  </si>
+  <si>
+    <t>Proposed research is innovative; developing a robust and informative RNA-protein interactome network map is a highly demanding challenge in the field; proposed approach is mostly logical; limited data availability and variability among the available experimental datasets and cell types could be a caveat</t>
+  </si>
+  <si>
+    <t>Scope and timeline are realistic, and proposed activities seem feasible; involvement of undergraduates is admirable, but the primary workforce (except help from a staff scientist from Boeynaems lab and support from NCEMS) being all undergraduates is somewhat concerning for timely completion of the project</t>
+  </si>
+  <si>
+    <t>Proposal aligns well with the goals and scope of NCEMS; appropriate data sources are identified, but the limitations are not discussed adequately; the proposal does not consider the variability among available datasets for the same mRNA interactions; RNA structural determinants should also be considered while predicting the RNA fate upon genetic perturbations</t>
+  </si>
+  <si>
+    <t>Highly collaborative project; admirable team effort; will use publicly available datasets; however, given the multitude of variables and factors associated with RNA-protein interactome and discrepancies among experimental datasets produced from different labs, it would be challenging for reproducibility; project deserves the benefit of the doubt though</t>
+  </si>
+  <si>
+    <t>The proposal is well-written and comprehensive and presents a clear and persuasive rationale for research activities to develop a robust and informative mRNA-protein interactome network map that can assist in predicting the effects of genetic changes at the mRNA level. The proposed activities are innovative, and their outcomes could benefit a wider community beyond the mRNA-protein interaction fields. The scope and timeline appear realistic and achievable. This proposal leverages the skills and expertise of well-qualified principal investigators, enhances collaborative efforts to conduct research activities, and trains new generations of researchers, aligning well with the scope and goals of an NCEMS synthesis project. The proposed tools and strategies are legitimate and achievable, and with the support of NCEMS's technical and intellectual resources, the proposal promises the timely completion of the proposed activities.
+However, the limited availability of mRNA-protein interactome datasets and lab-dependent variations and discrepancies among the experimental datasets could be a loophole and should be considered seriously. It is unclear if the proposal exclusively focuses on the K562 cells; variability among cell types may present a challenge. While the involvement of early-career researchers is admirable, the primary workforce of the project, mainly three undergraduates with partial support from a staff scientist and NCEMS staff support, raises concerns about the time and effort required for the timely completion of the proposed research activities. The project could benefit from considering RNA structural factors in addition to sequence perturbations when predicting the RNA fate associated with genetic perturbations. Nonetheless, overall, the proposal is convincing and feasible and aligns well with the scope of a synthesis project, with strengths outweighing its weaknesses. My enthusiasm for this proposal is high.</t>
+  </si>
+  <si>
+    <t>The main research questions are innovative and the general strategy is sound. If succeeded, the project will generate new tools and resource that are valuable for the research community . However, some key details in the approach are not clearly defined. E.g. what are the set of linked features and the normalization method (Aim 1.1) they plan to test. While it is understandable that these aspects will be refined as part of the project, the lack of examples or a clear plan/method to identify these parameters raises concerns about whether the proposal is sufficiently derdeveloped in this stage.</t>
+  </si>
+  <si>
+    <t>As mentioned above, identifying a viable linked feature and a suitable normalization method is critical not only for establishing the methodology in Aim 1 but also for the overall success of the project, as several subsequent aims depend on this method. Without additional details or preliminary considerations, it is challenging to evaluate the feasibility of the approach within the proposed timeframe.</t>
+  </si>
+  <si>
+    <t>The proposal clearly outlines a synthesis project, identifying all relevant public data sources. In this regard, it is well-aligned with the mission of the NCEMS center. The proposal also relies on various other types of data such as those from IP-MS, proteomic, biomolecular condensate, yet there is little discussion of their individual limitations and how these might impact the study's outcomes. </t>
+  </si>
+  <si>
+    <t>Commitments to generate open source tools and publically available database are indicated in the proposal.</t>
+  </si>
+  <si>
+    <t>This proposal aims to develop tools to integrate diverse RNA-protein mapping data to construct transcriptome-wide maps of mRNPs. The team further proposed leveraging these resources to derive biological insights through machine learning. Overall, this is a solid yet ambitious proposal with the potential to advance our understanding of RNA-protein interactions and their functional consequences. Key strengths include innovative questions, well-conceived overall strategy, and the potential to contribute to multiple disciplines through maximizing the use of existing genomic data. Additionally, the project aligns well with NCEMS's mission. The team is well-qualified, with complementary expertise across three labs.
+Areas for Improvement:
+Some methodological details, particularly regarding the selection of linked features and the normalization method (Aim 1.1), are not clearly defined, raising concerns about the feasibility of ahieving the goals within the proposed timelines. While these aspects are expected to be refined during the project, the absence of preliminary considerations and an approach to identify them is a concern. Additionally, the proposal does not sufficiently address the potential limitations of various data types beyond the RNA-protein map. There are also concerns about the reliance on undergraduates for key tasks, as they may require significant training before attaining the necessary level of independence to contribute effectively. Providing a clear plan for training and mentorship could help mitigate this risk</t>
+  </si>
+  <si>
+    <t>Elucidating the Role of Disordered Proteins in Cellular Adaptation</t>
+  </si>
+  <si>
+    <t>Strengths: 
+1. The evolution of protein sequences to adapt to environmental  conditions involves the complicated interplay of many biophysical,  genetic, and evolutionary processes and is clearly an emergent  phenomenon involving molecular/cellular processes. 
+2. Novelty in 1) leveraging metagenomic datasets in which  sequence distributions potentially vary with environmental  conditions, 2) coupling these DNA sequence data with protein  structure/biophysical property prediction, and 3) using AI/ML to  gain insights. 
+Weaknesses: 
+1. The approach suffers from the "house of cards" problem. While  the individual prediction algorithms such as AlphaFold3 or MD are  very impressive, they are not perfect. But more importantly  predictions from one algorithm, such as AlphaFold3 are fed into  another, such as Metapredict, whose output is fed into a third, such  as ALBATROSS or MD, and so on. The errors would propagate and  potentially amplify and it would be important characterize the  overall accuracy of the algorithm in predicting biophysical  properties of the proteins. Given that these proposals are limited to  computational work, this can be accomplished by applying this  pipeline for proteins whose structure/domains/biophysical  properties have been previously empirically characterized ("ground  truth") and determining the success rate. No such validation of the  proposed pipeline has been proposed. 2. The proposal is overselling its goals. Activity 3 aims to "uncover  the molecular principles governing adaptation of IDRs to diverse  environmental conditions." It appears that the study assumes that  that function would be conserved across environmental conditions  and evolutionary time. This is too strong an assumption.  Phenotypes could be conserved (or not) even if the individual  proteins have different biophysical properties in the different  environmental conditions by compensatory effects in other  processes, such as gene regulation or the function of other  proteins. Evolutionary capacitors, for example, are known to buffer  environmental insults.  
+3. In the absence of empirical data about function or selection, one  could potentially use population genetic signatures of selection  (McDonald-Kreitman test etc) to determine whether the IDRs were  evolving or not if it were possible to cluster conspecific sequences.  But no such approach has been proposed. 
+Miscellaneous: This project could be considered mesoscale or not  depending on whether the properties of individual proteins are  considered mesoscale</t>
+  </si>
+  <si>
+    <t>It is proposed that 4 papers, representing the creation  of an IDR database of 52K proteins, and 400K MD simulations,  multiple AI/ML approaches, would be produced in a 24-month  timeline. While a large team has been assembled, the scope seems  to be on the edge of feasbility, especially since each aim depends  on the previous one.</t>
+  </si>
+  <si>
+    <t>The project would synthesize information primarily  within the Ocean Gene Atlas v2.0 metagenomic dataset but also the  datasets implicit in the training of the various AI/ML models being  utilized. The data sources are explicitly identified.</t>
+  </si>
+  <si>
+    <t>Commitment to team: yes. Commitment to open and  reproducible science principles: nothing explicit has been stated  about data/code sharing and reproducibility (publishing software  containers etc).</t>
+  </si>
+  <si>
+    <t>This is an innovative and important project that fits  NCEMS's remit. However it has the moderate weaknesses of not  proposing any method to characterize the accuracy of the pipeline  in predicting biophysical properties and not really addressing the  question of adaptation raised in activity 3.</t>
+  </si>
+  <si>
+    <t>The variablity among disordered regions for organisms living in different extreme conditions has strong potential to help to determine sequence features that correlate with IDR regulation.  The proposal bring significant innovation to a significant question in the field.</t>
+  </si>
+  <si>
+    <t>My major concerns include: the reliabilty of coarse grained models to address changes in environmental conditions (e.g. is salinity accurately modeled), the reliablity of identifying homologues given the proposed ability of enviornmental factors to influence sequence composition, how well external salinity is correlated with the salinity in the cell's interior (what fraction of organisms are osmoconformers)</t>
+  </si>
+  <si>
+    <t>I had some concerns about the accuracy of protein annotation across such a wide range of organisms, having found cases of IDRs being weirdly annotated in some organisms.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not particular addressed. It would be easy to make sure this is incorporated, and the goal of rapid publication sort of addresses this. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overall the proposal is quite strong, with an innovating approach to connecting protein environment and function.  The combination of sequence analysis and simulation is sure to yield insight into the role of IDPs in protein adaptation.  For example, specific hypothesis derived from the sequence analysis can be tested with simulation.  However, the need for simulations as such a large scale was less clear. </t>
+  </si>
+  <si>
+    <t>The proposed work could be truly transformational except for one major weakness: pressure. The investigators seem to be entirely ignoring the massive impact that the varying pressure of the ocean has on protein structure/function, a factor that we are only beginning to understand. The predictive models that will be the first step in their identification of IDRs have all been trained on room-pressure structures. We simply don't know enough about pressure as a thermodynamic contributor to protein structure/function for the predictions to be reliable. What we do know is that pressure tends to eliminate void space (see works of Roche and Royer) and that the lone extensive analysis of pressure effects on a proteome (see Moran PRX Life 2024) showed that there are significant structural rearrangements of proteins in response to pressure, broadly speaking, not just for IDRs. If the IDR predictions are inaccurate, then ALL of the work that follows will lead to spurious conclusions. In fact, the applicants admit that they can't include pressure in the simulation work due to the lack of validated CG models. I'm surprised that they feel confident in ESMFold or AlphaFold3's ability to accurately predict disorder for proteins that have evolved to handle high pressure. Great ideas in this proposal, but this fundamental weakness means that the entire project and all the resources dedicated to it may lead to conclusions, models, etc. that are just flat-out wrong.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assessing how realistic the timeframe is for the proposed work is outside my expertise. The goals seem appropriate and the timeline is well-described. </t>
+  </si>
+  <si>
+    <t>The synthesis power of the proposed work seems very strong to me (with the misgivings noted above), and the data set seems an ideal one for the proposed insights.</t>
+  </si>
+  <si>
+    <t>This is not explicitly addressed, and I lack the expertise to assess this aspect based simply on reading the methodology proposed. All that is said about dissemination is that they will publish findings. Nothing about making the tools developed or data (structure predictions, trajectories, analytical outputs, etc.) broadly available or anything like that.</t>
+  </si>
+  <si>
+    <t>This proposal aims to unveil environmental adaptation of IDRs from genetic data of marine organisms sample from a broad range of environments. This is an ambitious aim, and the combination of methods proposed is cutting-edge. The investigator team has considerable expertise in IDRs, especially with respect to biomolecular condensates. The data set is an untapped resource for understanding protein structure/function, so that aspect of the proposal is quite exciting. There are several weaknesses, unfortunately, that drive my major skepticism for the reliability of the insights that would result from the proposed work. Most importantly, the proposal fails to recognize the massively complicating factor that pressure will play in the data set, the scientific questions posed, and the methods they propose to use. They don’t plan to simulate pressure due to the absence of a pressure-validated course-grained model, yet they fail to realize that the algorithms they will use to predict intrinsic disorder in the first place are not parameterized in any way to account for the pressure effects on protein structure. The IDR prediction from genetic data is the first step in the entire project, so even a moderate error in that prediction will likely cascade into a host of spurious outputs. I would feel a little bit better about a protein-based analysis of this data set if the goal were to study well-structured proteins with high homology, as there is at least ample data for comparision of well-folded proteins from extremophiles in the PDB, but the plan to examin IDRs, for which the predictive models should not be trusted for extremophilic proteins, is especially worrisome to me.</t>
+  </si>
+  <si>
+    <t>Intrinsically disordered proteins/protein regions (IDRs) are a relatively novel phenomenon of the condensates area of molecular biology. The proposal is an atempting to uncover universal features that induce IDR adaptation using Marine metagenomics and metadata. The research is addressing phenomena at the mesoscale level. This topic is very important and innovative as this is a newly emerging field of cellular biology.  
+Their methodology seems practical and justified. Many of the computational programs mentioned to be used are recently produced by members of the team, so the methods are emerging practices and the personel are fit for the project.</t>
+  </si>
+  <si>
+    <t>Aim 1 has only five people assigned, but is said to take six months even though it is to be the base of their entire scientific framework. Aim 2 also has five people and is expected to take 12 months. Aim 3 has seven personel dedicated to it, and is expected to take one year. I would be concerned about the length of time proposed since it seems much of their Activities build off of the previous one's success, but they have 17 personel working on this project and even their "trainees" are considered experts in the fields of the Activities they are assigned to.</t>
+  </si>
+  <si>
+    <t>Yes, this is explicitly a data synthesis project. They clearly laid out the three data sources they would be using and computational limitations were appropriately acknowledged.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">They state that one of the outcomes of the project will be a database of IDRs, which is a source of Open Science. The methods with which they will be performing their science use primarily open source materials and are likely reproducible, but that can not be determined exactly. There is no direct mention of a commitment to open, team, and reproducible science principles, or statement of open science. However, in the "Proposal Narrative" provided to proposers, it does not require that any open science compliance statement be provided in the Proposal Narrative directly. This creates a very difficult situation for evaluation of this section. This group seems to have a history of providing open source materials, and so it is likely they will continue this trend. </t>
+  </si>
+  <si>
+    <t>Intrinsically disordered proteins/protein regions (IDRs) are a relatively novel phenomenon of the condensates area of molecular biology. This field is becoming increasingly studied across fields as we begin to learn its importance in biological functions. The proposal is atempting to uncover universal features that induce IDR adaptation by: cataloging excessive amounts of genomics data into IDR data, observing IDR properties in different external contions with metadata in the form of salinity and temperature, mapping how the IDRs adapt in an atempt to engineer IDRs in the future, and creating a database of these IDRs and the aformentioned information. This proposal hits the mark on all of the scientific a methodological requirements for this NOFO, and the Lead and Co-Leads are established in their respective fields. 
+As this type of proposal is quite unique, it is difficult to know who you will get as a reviewer. The proposal would have benefitted from an example known IDR functions (the C. albicans CO2 response paper is quite interesting) to provide context for what they are capable of doing for organisms. This would have provided some needed contextual importance of the broader subject matter (IDRs) beyond the Ocean microbiomes. It would also have been useful to indicate next to the sub-activities the length of time you think each will take, or a summary table. It was difficult parsing how long the entire project would take based on your description at the end. Otherwise, the personel chosen for this are perfectly aligned to take on the task, and hopefully it will lead to improved understanding and possible increased databases of IDRs in other ecological contexts.
+   Additionally, reviewers were provided with the 2024 RFP and the 2024-2029 NCEMS Strategeic Plan, both of which are available online. Unfortunately, the RFP narrative requirements and what the Strategic Plan and Objectives/Scope of the RFP are not entirely aligned. This proposal stuck to the RFP Narrative Requirements 1-14 to a T, but the review template has additional sections that are more aligned with the Objective/Scope which is not entirely a fault of the proposal.</t>
+  </si>
+  <si>
+    <t>Multimodal Single-Cell Frameworks for Cell Lines with Extensive Multi-Omics Data</t>
+  </si>
+  <si>
+    <t>The proposal addresses an important question of comparing DNA, RNA, and protein levels within the same cell. Multimodal data analysis has significant potential to advance knowledge of how DNA, RNA, and protein levels vary across independent cells.. One limitation is that some of the datasets from Dr. Brunk's lab are unpublished. A key feature of the proposal is analyzing multimodal data that simultaneously assess two of three modalities (DNA, RNA, protein) in 7 model cell lines and integrating these datasets with numerous other datasets in these cell lines such as bulk sequencing and proteomics and PERTURB-seq. However approaches to measure RNA and protein such as ECCITE-seq only can measure a limited number of proteins. The cited ECCITE-seq dataset looks to have analyzed RNA content associated with ~50 cell surface proteins. The limitations on the matching of the protein level to DNA or RNA was not sufficiently addressed. The PI mentions FACS+FISH+4i datasets to monitor DNA and  protein levels but there are no references or description for this technique</t>
+  </si>
+  <si>
+    <t>Goals and timeline are reasonable</t>
+  </si>
+  <si>
+    <t>Data sources are appropriately listed. The proposal clearly demonstrates a synthesis project. One weakness is that five key matched datasets generated by Dr. Brunk are listed listed as being in manuscripts in preparation or under review and were not available.</t>
+  </si>
+  <si>
+    <t>There clearly is a commitment to team science. The nature of the proposal focuses on reproducible science by focusing on 7 cell lines. There is mention of making tools, findings, and pipelines broadly available, but how this will be achieved was not explicitly explained. Judging the commitment to making the data open is difficult to assess as several key datasets are listed as being in manuscripts in preparation or under review. Preprints describing these datasets would have gone a long ways to alleviating this critique.</t>
+  </si>
+  <si>
+    <t>This is a good proposal from an outstanding team of investigators. It addresses an important question of exploring levels of DNA, RNA and protein in single cells to determine their relationship and variaibility. The author propose to use 7 cell lines with ample bulk and single cell perturbation datasets. They propose  modeling using data that simulataneously measure two modalities (DNA and RNA, DNA and protein, mRNA and protein). They make a good case for use of NCEMS support. Weaknesses include a lack of description of unpublished datasets that are key for evaluating feasibility of the proposal. It's not clear how the PI is measuring DNA and protein. The limited connection of the RNA and protein levels (ECCITE-seq dataset only studied ~52 cell surface proteins) and how the authors will be able to model DNA, RNA and protein levels with a limited set of cell surface proteins was not addressed. How the authors are studying DNA and protein was also not sufficiently described. Overall, these strengths and weaknesses were balanced and resulted in moderate enthusisam for this proposal.</t>
+  </si>
+  <si>
+    <t>The investigators aim to crate a benchmarking dataset for multimodal multi-omics data from matched cell types. The rationale for this project seems to be that, while many methods exist to understand relationships between multimodal datasets from unmatched cells, there are far fewer from matched datasets and this limits downstream biological analyses. While the effort to perform integrated analysis across multimodal datasets remains challenging and thus there is a crucial need for developing these resources and tools in gene regulatory analyses, it is unclear what the main advance or advantage being proposed in this proposal. It would be useful for the investigators to better spell out the biological questions that necessate these approaches. Additionally, while there is very useful details on the datasets and backgrounds of the team, there is little detail as to how the analyses or developments of novel methods will be performed.</t>
+  </si>
+  <si>
+    <t>The assembled team has amble experience with these datasets, so the goals and milestones seem reasonable in the timeframe.</t>
+  </si>
+  <si>
+    <t>Yes, this is clearly synthesizing across many datasets that one or even two labs would have a hard time analyzing. The inclusion of various sequencing, imaging, and protein datasets requires more advanced synthesis techniques.</t>
+  </si>
+  <si>
+    <t>Good descriptions of making all the code, pipelines, and final databases pubically available after the project is completed. Will be an excellent resource for the community.</t>
+  </si>
+  <si>
+    <t>This proposal aims to use a well-curated list of datasets across different gene regulatory processes to create a benchmarking dataset for matched multimodal multi-omics datasets. While I think this is generally a useful aim, it is unclear from the proposal what this dataset is precisely aiming to benchmark and which biological questions would be most aided by the creation of this resource. Additionally, it would be useful to have more details on the statistical approaches proposed to create their models and the novelty of such approaches. However, it is clear that the assembled team is quite strong with a great track-record of applying such datasets towards interesting biological questions, so the resources that would come out of this work would be very useful to the community. A strength is also the aim to make the harmonization code, pipelines, and concepts publically available to the community, which would be extremely useful for future such efforts.</t>
+  </si>
+  <si>
+    <t>This propsal does not explcitly address " emergent phonomena, it doses aim to integrated the multi scale interacaction in molecular and celluar systems. The novelty of the proposal focused on single cell approach within homogenized cell line system and the frame works for multi-layered regulation which will benifiting the broader community. 
+The methodology appears clear and logically organized. However, it would be beneficial to provide some more detail on how the research standardizes the metadata with a clear pipeline description of how this pipeline and the team will manage the multi-cell interaction between the different cell lines, as most of the proposal has focused on single-cell lines currently.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The propsal is stongly supported by preliminary data, and the goal of the project and the  timeline is fasible. </t>
+  </si>
+  <si>
+    <t>This project is not a synthesis focus. As the described, the multi-omics data has already collected, the proposing project is focused on utilized the current data and generalized the frameworks into a model pipeline.  </t>
+  </si>
+  <si>
+    <t>The proposal indicates the they will deliver dockerized piplines and made broadly accessible to the community. Also they mentioned that the output of the project can be access by over 1000 students annully with the biochemisty course with should aligned with the open science principle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The proposed project focuses on utilizing existing data and generalizing the framework into a model pipeline. The novelty lines in the single-cell approach within homogenized cell lines, offering multi-layered regulation. The project will benefit the broader community with the delivery of a dockerized pipeline. The methodology is generally clear and logical, though more detail on metadata standardization and multi-cell interactions would be helpful. The project is strongly supported by preliminary data and the goal and timeline are feasible. </t>
+  </si>
+  <si>
+    <t>The goal to combine data of different cellular layers is important and innovative. Their approach of employing single cell analyses of the same cell line will likely enable cleaner results than that of various origins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This integrative analysis is not my expertise and therefore I do not have experience with its time frame, but the proposed timeline appears reasonable. </t>
+  </si>
+  <si>
+    <t>This proposal is clearly a synthesis project and the data sources are explicitly identified. However, the limitation of the proposed cell lines A549 and COLO320DM lacking matched data across all 3 layers is not discussed.</t>
+  </si>
+  <si>
+    <t>The educational impact of this proposal is admirable, and the team approach is clear. However, the output of their findings is not clear, and whether the findings will be open-source is not stated. This is a major weakness in the proposal.</t>
+  </si>
+  <si>
+    <t>Strengths: This proposal meets many of the goals of NCEMS. The proposal describes an innovative tool that will unify currently available omics data within specific cell lines to understand how each of these cellular layers influence each other. The tool has useful implications for many scientists. This approach requires wide ranging expertise, and the group has curated an accomplished team with a mixture of early and late stage PIs across many institutions to meet their goals. Additionally, trainees at varying career stages both in the research lab and classroom will also benefit from learning the skills proposed here.
+Weaknesses: Despite the innovative approach and clear impacts, the key weakness in this proposal is the lack of a well defined output with open availability. Will the proposal result in an open source database of their findings? Will the findings be released in a research manuscript? NCEMS requires that these proposals result in one of their defined outcomes, and it is not clear that this proposal will accomplish that goal that. Additionally, as a note, calling the cell lines "primary cell lines" is misleading because many are cancer cell lines that have been grown for many decades (i.e. HeLa) rather than recently collected tissue that is not immortalized.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The proposal explicitly focuses on emergent phenomena in molecular/cellular biosciences, and its goal is to leverage existing data to develop model-specific multimodal frameworks that integrate single-cell sequencing and imaging data from the same cell line, enabling unified representations that capture simultaneous measurements of DNA, RNA, and proteins within individual cells. These frameworks will likely provide a clear and more detailed understanding of the cell-to-cell heterogeneity that drives cell population diversity. 
+This project is novel as it integrates matched single-cell sequencing and imaging data from the same cell line, unlike current efforts that focus on unmatched data. It uses advanced methods like variational autoencoders, graph neural networks, manifold alignment, and canonical correlation analysis to infer relationships across DNA, RNA, and protein layers. This provides new insights into cellular heterogeneity and regulatory processes.
+The methodology is grounded in robust computational and statistical practices, utilizing established tools (e.g., Harmony, Seurat) and emerging techniques (e.g., late integration methods). </t>
+  </si>
+  <si>
+    <t>The timeline is realistic but adding buffers, especially for data harmonization and experimental validatio, will enhance feasibility and success rates.</t>
+  </si>
+  <si>
+    <t>The proposal clearly demonstrates a synthesis project by integrating diverse data types (including DNA, RNA, and protein measurements from single-cell and bulk sequencing, as well as imaging data), leveraging interdisciplinary expertise from bioinformatics, machine learning, network biology, and genomics, and developing unified frameworks and tools. The data sources are explicitly identified, and limitations (e.g., data fragmentation, alignment challenges) are appropriately acknowledged, demonstrating a realistic and well-considered approach to data use.</t>
+  </si>
+  <si>
+    <t>The proposal clearly demonstrates a commitment to open, team, and reproducible science principles by planning to share data and tools openly, ensuring transparency and facilitating external validation. It emphasizes interdisciplinary collaboration, combining expertise from bioinformatics, machine learning, and biology to tackle complex challenges effectively. Additionally, it outlines rigorous methods for reproducibility, including detailed documentation and validation of workflows, ensuring that results are reliable and can be reproduced by others.</t>
+  </si>
+  <si>
+    <t>The proposal focuses on developing innovative multimodal frameworks that integrate single-cell sequencing and imaging data from the same cell line. This approach enables unified representations of DNA, RNA, and protein measurements within individual cells, offering deeper insights into cell-to-cell heterogeneity. Its novelty lies in using matched data, unlike current efforts with unmatched datasets. Advanced methods like variational autoencoders and graph neural networks are employed to infer relationships across biological layers, providing new perspectives on cellular heterogeneity and regulatory processes.
+The proposal could benefit from leveraging both matched and unmatched data to enrich the dataset, providing a broader context and more comprehensive insights into cellular heterogeneity. Additionally, more detailed planning for scalability and resource allocation, including contingency plans for unforeseen delays, is needed to manage the increased data volume effectively.</t>
+  </si>
+  <si>
+    <t>From Image Data and Biophysical Simulations to Principles of Mesoscale Organization Through Integrated Transfer Learning</t>
+  </si>
+  <si>
+    <t>The authors want to understand mesoscale celluar organization. Their approach seems novel. My major concern is that the questions they are asking and the methods they are proposing to develop are quite vague. For example, the atuhors ask “what role do mesoscale interactions play in determining the morphological and physico-cemical properties of …”. It is not clear what this question means. What do the authors mean by “interactions” Do they just mean physical proximity? Morphology is complex and it is unclear if the authors plan to quantify morphology based on some TDA like statistic or something else.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The timeline seems a bit optimistic but it may be enough for a proof of concept. Albeit, it is not exactly clear what they are proposing to answer (scope) or how they are proposing to do it (methods). </t>
+  </si>
+  <si>
+    <t>The authors have identified a number of relevant datasets but it is not clear if they will be able to get access to that data. The authors are requesting support to help scout datasets. I doubt NCEMS will be able to provide this support effectively and efficiently.</t>
+  </si>
+  <si>
+    <t>In Broader Impacts the authors suggest their work will be made publicly available but no details are provided. It is unclear what would be produced by this research or how it would “empower researchers”.</t>
+  </si>
+  <si>
+    <t>This is an interesting proposal that definitely seems inline with the goals of NCEMS. My major concern is that the goals of the project are vague and the methods seem to be missing key details.</t>
+  </si>
+  <si>
+    <t>The work group focuses on the intepretation of the mesoscale cell biology through a statistical physics point of view. They use the high volume image data with spatial and temproal resolution towards this study. The output will yield three major complex mesoscale phenomena in cells. However, the justification and choice of data for each specific biological question is not well defined. The instrinsic connection or hypothesis for such connection is not well justified. Furthermore, there was no preliminrary work supporting these hypothesises. Finally, details of the approaches are missing.</t>
+  </si>
+  <si>
+    <t>The overall timeline of the project is feasible. However, I am not sure what would be implemented in component 5c, the intrgration and synthesis.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the team will have access temporal data from the Allen Institute for Cell Science and CZI. However, there are multiple cell lines data, it is unclear how the team will take consideration of the cell type heterogeneity towards their investigation in the general principles for the mesoscale structures. Also, there is no existing publication from the team based on the data from Allen or CZI. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">identifying the generality of subcellular mesoscale structures requires innovative perspects from Physics. The work group proposes novel approaches based on the high-resolution imaging data. However, the reviewer's enthusiasm is dampened by the lack of details for scientific hypothesis and approaches. </t>
+  </si>
+  <si>
+    <t>These questions are timely and align with current challenges in cell biology, particularly in leveraging the massive volumes of imaging data. The use of GW distances to develop transfer learning algorithms is novel.
+Focus on nucleus related components provides a tangible outcome for this project but the scope and implications outside of these example cases are not clearly described, nor is rationale for starting with the nucleus related components. The outcomes suggested are very broad but how the research team gets there from the nucleus and its current abilities is unclear.
+The methodology is moderately clear. The researchers describe more about the steps that the data will be taken through, however, there is a lack of description of the data types, especially related to simulation, and a lack of consistency of the data types across the three examples.</t>
+  </si>
+  <si>
+    <t>Two years is an appropriate timeline but there is a lack of detail in the timeline to ensure timely progression of the project as well as which team member lab is doing which aspect. More micro milestones will be useful, as well as if the 3 examples will be done in tandem or sequentially.</t>
+  </si>
+  <si>
+    <t>There is weakness in the data sources used, especially related to in silico simulation. It is explicitly said that more data scouting would need to be prefered, which while appreciated in the sense of a limitation discussed, there is not a cohesive description of what data will be used. OpenNucleome and the 4D nucleome project are discussed, for example, but one of those is a software and the other has data in it that is not necessarily simulation related.
+Examples 2 and 3 do not mention simulation data, which is a major premise in the description of the project (and in the title). Ultimately, the authors could be more specific on what data they will use so that there is confidence in the feasibility of at least one example working, and a connection to how this can be extrapolated to other biological systems since a main goal of the work is to develop a broad use framework.
+There is a synthesis discussed between data types and scales, but enthusiasm is dampened given the lack of clarity, availability/type/insight to achieve from, and use of the data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> It is mentioned but there are no tangible outcomes of how the data will be open. Mention of GitHub, Open Science Framework, etc. would have given confidence of a plan to make the workflow/framework available. Also, what constitutes the framework that will be available? Scripts, a GUI interface? Where will individuals access the curated database? How will individuals interact with the validated models?? </t>
+  </si>
+  <si>
+    <t>The proposal addresses critical, current challenges in leveraging large imaging datasets to uncover mesoscale cellular organization. Its use of transfer learning, specifically incorporating GW distances, is both novel and promising.
+While the proposal outlines a broad strategy for data integration, it lacks clear details about the specific data types and sources that will be utilized, particularly for simulation data. A more detailed plan for data use and curation is essential to instill confidence in the feasibility and scalability of the approach.
+The methodology for implementing the project is only moderately clear, with insufficient detail regarding the timeline, milestones, and team roles.
+While the proposal aspires to create a broad-use framework, the specifics of how this framework will be made accessible are not well-defined. The lack of concrete plans for open science practices—such as use of GitHub, Open Science Framework, or curated databases—reduces confidence in the project’s potential impact and usability.</t>
+  </si>
+  <si>
+    <t>Transposable elements and the emergence of genomic innovation</t>
+  </si>
+  <si>
+    <t>The proposed research concerns an emerging advance of knowledge regarding transposable elements, which hold promises to reveal the details of genomic regulatory landscape innovation. I find the relevance of the proposal very high. On the other hand, I find the novelty of the proposed research slightly lower, just because I feel the proposed research is a logical extension in the era of T2T genome-functional genomics. In terms of the approach, I have some reservations about their 'repeat aware' pipeline. As written, it is unclear how much of the MMR could be parsed through Allo. Therefore, I am slightly concerned that their approach cannot access all repetitive regions of the genome. The specific deliverables from the phase 2 is unclear beyond the posited associations. Nevertheless, this is an exciting and timely proposal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The proposed research is well planned and I have confidence that the collaborative team will generate deliverables within the proposed timeframe, especially with the provided computational resources. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data to be used in the proposed research are all identified. There may be some additional limitations as I mentioned in the section A. Even though this is an exciting genomic and functional genomic proposal, I find the synthesis component slightly lacking. This is because all the members of working group are already working in the field of transposable elements, and the proposed research is an in-depth application of new data and methods rather than opening a new direction of research. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The working group indicated that all data and mapped resources will be publicly available, but did not specify how they intend to do so (which would be non-trivial given the vast amount of data), and I don't see specific budget allocated for doing so. </t>
+  </si>
+  <si>
+    <t>The proposed research aims to investigate how transposable elements (TEs) contribute the evolution of novel functional genomic elements such as transcription factor binding sites (TFBS), enhancers and protein-coding sequences. A key knowledge gap driving this research is the limitation that current functional genomic data have used short read sequencing, thereby not able to access highly repetitive regions of the genome. To address this, the working group proposes to use T2T assemblies and probabilistic methods to resolve multi-mapped reads. While this is a timely and relevant proposal, the deliverables ultimately are descriptive, and the synthesis across different discplines was lacking (though it is an excellent functional genomic study). Nevertheless, the proposed research investigates a timely and important problem in functional genomics, their plans are detailed and feasible, and the proposed budget appears to be appropriate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reprocessing of the 70,000+ datasets to account for multiple mapped transposable elements will advance our knowledge of how these elements contribute to the evolution of new regulatory elements. The proposal uses established, rigorous tools to reprocess the datasets. The rigor of phase 2 could be improved with examples how these comparative genomics approaches have successfully identified new regulatory elements. </t>
+  </si>
+  <si>
+    <t>The timeline is reasonable and justfied well.</t>
+  </si>
+  <si>
+    <t>The 70,000+ datasets that will be reprocessed is a clear synthesis project. All the datasets are clearly identified and acknowledged.</t>
+  </si>
+  <si>
+    <t>The PIs outline how all processed data will be publically available. The analysis pipelines will also be publically avaiable. In addition, the PIs expliciltly request funds to publish open access.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Our understanding of how transposable elements contribute to the evolution of new regulatory elements is limited due to the challenges of mapping repetitive transposable elements to genomes. Multiple mapped reads have been omitted from most studies, leading to an under annotation of transposable elements. The PIs propose an excellent use of NCEMS resources to reprocess thousands of datasets using repeat-aware pipelines. This is a clear match to NCEMS aims to reuse existing data. Another strength of this proposal is the repeat-aware pipelines already exist, so data collection and reprocessing can begin immediately by NCEMS staff. The newly processed datasets will certainly provide new insight into how transposable elements generate new functional regulatory elements. The only minor weakness is the experiments outlined in phase 2 are only briefly described. An example of how these comparative genomics approaches across species have resulted in identifying new functional regulatory elements would be helpful. The proposed working group has the expertise needed to achieve the goals.  </t>
+  </si>
+  <si>
+    <t>The proposed two-phase project aims to reprocess public genomic data using repeat-aware analysis pipelines and T2T pangenome assemblies to account for transposable elements. This has significant implications in the field. The PI has published methods capable of handling multi-mapped reads and identifying new TF binding sites. With the new information gained from this project, it can spark numerous emerging researches.</t>
+  </si>
+  <si>
+    <t>The project requires large computational resources. The preliminary data consists of 1% of the planned data processing and took several weeks with local resources. The aim of this project is to reproces all the transcirptional and translational data, which is a bit ambitious.</t>
+  </si>
+  <si>
+    <t>Good demonstration of collaborative effort that requires expertise from multiple labs. The majority of the effort will be performed in the PI's lab. Data sources have been clearly identified.</t>
+  </si>
+  <si>
+    <t>The processed data will be made publicly available.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is a very compelling and ambitious proposal to reprocess genomic data to account for transposable elements, and their connection to functional elements. It will address an important question and at the right time when T2T projects provide new genome assemblies. The method used in this proposal has been published, and has a well-reasoned plan that requires expertise from multiple teams and strong support from NCEMS. The proposed project is a little bit too ambitious, but once delivered, it will serve as a valuable resource for the field. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transposable elements (TEs) are a challenge - they are clearly important for evolutionary innovation, but they are also notoriously difficult to study because they are, by nature, repetitive and distributed throughout host genomes. This proposal aims to re-analyze available data to characterize the role of TEs in variation in gene expression through altering regulatory architecture of gene expression. There is ample data available and the team presents a rigorous approach. </t>
+  </si>
+  <si>
+    <t>The timeline is discussed and clear. It does seem ambitious for a 2-year time period, but this depends on the timeframe for analyzing the 70,000+ data sets available. The applicants do suggest that the project is "shovel ready" which provides some confidence that they can hit the ground running and make good progress quickly.</t>
+  </si>
+  <si>
+    <t>My main concern here is that the data available is, by nature, haphazardly collected. Sources will be different genotypes, sexes, etc. so the reference telomere-to-telomere genome approach won't necessarily deal with that variation appropriately. The investigators also mention utilizing pangenomes, but it isn't clear how all of these aspects would fit together.</t>
+  </si>
+  <si>
+    <t>Open science is mentioned in the "Outcomes" section, but it is briefly and does not permeate the rest of the proposal. However, the sharing of pipelines, data, etc. is appropriate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This proposal aims to determine how transposable elements contribute to genomic innovation through a comprehensive reanalysis of available genomic and transcriptomic data for vertebrates (mostly mice and humans). Strengths include the research team, a clear demonstration of feasibility via a pilot analysis of a subset of the available data, and an excellent premise: TEs likely are an important contributor to genome innoviation but are often overlooked because they are difficult to pin down. The proposal describes two complementary approaches (T3E and allo) for identifying insertions and determining their association with transcriptional changes. 
+The proposal was strong overall. It could be strengthened by better spelling out the way in which gaps in the data (data types: transcriptomic, CHiP, genetic variants) would be handled. Another are for improvement is a clearer picture of the timeframe to achieve these results given access to NCEMS resources. </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Searching the Crosslinking Mass Spectrometry Universe for New Protein-Protein Interactions</t>
+  </si>
+  <si>
+    <t>The proposal targets an important frontier of biology (++). The proposal seeks to revisit and homogenize the analysis of a select set of deposited cross-linking MS datasets.</t>
+  </si>
+  <si>
+    <t>The workflow described for task A appears to be tractable with the resources provided. Task B appears to be rather open ended.</t>
+  </si>
+  <si>
+    <t>The proposal relies upon deposited data. While noting some of the differences in deposited data format and source, the proposal does not address the issue of data quality within the existing databases. There is no specified procedure to vet inputs.</t>
+  </si>
+  <si>
+    <t>This proposal provides a clear plan to use open-source data and to provided updated versions of these datasets – improved by the proposed work.</t>
+  </si>
+  <si>
+    <t>This proposal 
+The objective of this project is to improve data infrastructure around protein protein interactions as assess by cross-linking MS. This is an accepted method for this purpose generating meaningful datasets. It is however a niche method with a small but relevant community. As such there are less than desirable metadata and data treatment consistency. The project seeks to gather and harmonize this approach. The strengths of this project are the topic – at the forefront of metabolic network understanding. The primary weakness of this project is the small working group. The team is very strong and ideally credentialed for the proposed work, but does not feature complementary pieces which broaden the project and might create buy-in for the resulting database formats and tools. This appears a lot like a single / pair of investigator projects leveraging a community resource project.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This team seeks to further explore, at larger scale, currently avaibale XL-MS datasets to investigate not only protein-protein interactions but to interrogate more regional specific information that is available via XL-MS and not by other interactor studies (AP-MS, co-fractionation, etc). The team accurate idenfies an issue of re-using publically available datasets, as software tools have been limited for XL-MS, and many groups find data interrogation chanllenging. The project is extremely imporant although perhaps not novel. One issue is that the team indicates structural implications of the data, but that is not noted in the approach other than a "look and see" if residues are close by AlphaFold. One other concern is the focus on MS-cleavable crosslinkers.  Many of the legacy datasets use non-cleavable linkers (acrylamide), this should be a priority for the team as these data are very challenging for common users to analyze. My recommendation would be to prioritize this over a list of other species that are available. The functional assessment is likely overambitious based on this limited information.   </t>
+  </si>
+  <si>
+    <t>The goals and layout of the proposed project are reasonable however as noted above, there is some concern about the potential of exploring many different species and prioritizing this over other unique informatio that can be gleaned from focusing on Human or yeast datasets first.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The project seeks to address currently available data and to re-assess the informtation that can be obtained. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The team will use publicallya vailable data. </t>
+  </si>
+  <si>
+    <t>I believe that this project is very important and will be impactful to the proteomics and structural biology community.  Strengths and weaknesses are balanced, with significance being strong.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This project aims to wrangle the XL-MS data sets that already exist while also building a set of best-practices for data structures, annotation, etc. necessary for this incredibly powerful data to be accessible to the broader scientific community. Essentially, I see this as a project that NEEDS to be done for the promise of XL-MS to be realized. The approaches proposed for data curation/organization, etc. are not innovative in and of themselves, but that's appropriate because there are plenty of established ways to effectively build searchable databases. The main likely parts of the project where new tools may be developed will be the last portion wherein protein-protein interface identification and discovery will be involved. </t>
+  </si>
+  <si>
+    <t>This project is very doable in the proposed timeline, though the goal 3 aspects are necessarily poorly defined. It makes sense that definition of how information of protein-protein interfaces will be mined/explored must depend on how much of such information is available in the data once the data is curated and annotated</t>
+  </si>
+  <si>
+    <t>The proposed work will clearly synthesize data sets from various organisms and experimental approaches. Though the data sets are all from XL-MS, there is sufficient variability in the data sets in terms of source, cross-linker, etc. to necessitate challenging synthesis.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A mechanism for XL-MS data to be searchable and minable is a central goal. This would be a huge boon to the scientific community, not only for the data that already exists, but for the likely considerable expansion of such data in the future. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">This project seems doable and important. XL-MS is an incredibly powerful technique that is only becoming more powerful as experimental methods, instrumentation, and computational approaches advance. The size of the existing data is large and complex enough to warrant NCEMS help with unifying the data structures and establishing standardized practices for deposition now (as opposed to sometime in the future when there will be ever more data, making the job progressively harder). Most importantly, the existing data has huge potential to reveal transformative insights, and the establishment of standardization, public availability, and uniform usefulness of the data will build the foundation for XL-MS data to provide the worldwide scientific community with access to novel information about biology. </t>
+  </si>
+  <si>
+    <t>The proposal does not explicitly discuss the emergent nature of the research, though it can be inferred that the work will uncover protein-protein interactions that are otherwise undetectable when considering data collected differently (i.e. AP-MS). The innovation is to leverage structural insights from both crosslinking MS and structural predictions to describe PPIs in humans and yeast, and to compare the results to the robust PPI landscape that does not consider structural data. This work is important and has great potential to advance knowledge. For the most part, the methodology is clear, logical, and grounded in established research practices. Methodologies for Activities C and, to a lesser extent B, are not described at the same level of detail as Activity A and could be strengthened.</t>
+  </si>
+  <si>
+    <t>The researchers have allotted 6 months for NCEMS-assisted manual data curation of publicly available XL-MS data, which seems realistic given that one of the working group leads has expertise with the PRIDE database. The second phase of the project builds upon the first phase to bring in structural predictions as a validation metric. It is unclear if 6 months will be sufficient time to perform and analyze up to 15,000 pairwise structural predictions and the researchers have not provided what they anticipate will be the final number of pairs to investigate. Insufficient methodological detail was supplied to assess if 3 months is realistic to achieve Activity C.</t>
+  </si>
+  <si>
+    <t>The project is clearly a synthesis effort and will draw from at least 31 publicly available XL-MS datasets describing a total of 6480 total MS experiments. The effort to wrangle this data, curate the metadata, and re-analyze with modern tools is worthwhile. The researchers have identified the datasets clearly and have described the challenges to working with these datasets without manual curation, clearly indicating the need for NCEMS support.</t>
+  </si>
+  <si>
+    <t>The researchers will use publicly available data, clean it up and re-analyze, and repost the improved result. This is a great effort to support open, team, reproducible science.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The proposed work seeks to uncover protien-protein interactions in humans and yeast using publicly available cross-linking MS data, and to compare the resulting cross-linked peptide hits to structural models of the parental proteins. This work complements existing human PPI networks well as the current methods do not consider structural data and largely rely on affinity-purification MS. The existing PPI data thus may have a high rate of both false positives (lots of "sticky" proteins come down in an AP-MS experiment) and missing interactions (i.e. those that fall apart during purification). XL-MS provides an orthogonal approach, and the researchers use of protein structural predictions to validate their results is compelling. The researchers plan to re-analyze and re-post data to meet current quality standards is valuable, and the goal to incorporate all data into the Complex Portal is good. 
+The proposal could be considerably strengthened by further development of Activities B and especially C. For example, specific details on how the researchers will assess the structural models for compatibility with the XL-MS data would be appreciated (Activity B). Even better would be to also utilize existing experimental structure data, which is likely to be available for a large number of human proteins and complexes. Collecting this structural data is a task that NCEMS support could also be used for. Activity C is only very briefly described and it is not very clear what the method or outcome will be. This area merits further deveopment, however it is a minor goal compared to those in Activities A and B. </t>
+  </si>
+  <si>
+    <t>Intelligent metadata compilation to enhance the reusability and discoverability of mass spectrometry based</t>
+  </si>
+  <si>
+    <t>This team seeks to address a significant issues in the public availablity of mass spectrometry data, namelly limited to no metadata.  As a result, reanalysis or use of such public data has been hampered.  I find this to be an important area that is being addressed.
+The proposal is very text heavy, could be beneficial to see an example of an expected output metadata file.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strategy to start with bottom-up datasets is strong. Will expand if time permits, to other types of data, but establishing a standard for the community will be extremely impactful. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes  the initial development will be on 244 datasets. One question is, one the methdology is established, how many datasets do the team plan to process? How will they dissemenate their tool besides GitHub and publication? Do they anticpate fields to adopt this workflow? Outcomes are general, milestones may be better. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, the team is addressing this. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very important project that is much needed in the community.  The team is qualified to handle the project.  Some weaknesses noted above but strenghts outweigh. </t>
+  </si>
+  <si>
+    <t>The researchers propose an important task, but to me, the proposal as written does not quite get at an emergent phenomenon. The proposed outcome of getting existing data into alignment with FAIR principles is excellent and much needed in the scientific community, and will have the potential to advance knowledge down the line. The general process of developing workflows was clearly explained and will combine both raw data and textual data mining approaches.</t>
+  </si>
+  <si>
+    <t>The project goals seem reasonable and attainable - the proposed work encompasses several tasks, but the timeline is well organized. The proposal did not address potential roadblocks that may impede progress and/or how they will be navigated.</t>
+  </si>
+  <si>
+    <t>My view on synthesis involves bringing individual pieces together to result in something new, which could not be extracted from examining each piece separately. The proposed works develops a new curation process with a great output (in the form of integration with the existin PRIDE database, which will have the potential for something new, but the emergent knowledge is several steps removed. Data sources are clearly identified. Limitations due to missing metadata are acknowledged, but the impact on the overall output is not fully addressed. Limitations to the raw and textual data mining processes based on the data are also not directly addressed.</t>
+  </si>
+  <si>
+    <t>Open science is addressed with concrete actions (open-source software, licensure, open-access publications, etc.) and includes a plan for code dissemination on GitHub. Educational resources were also mentioned, but the form these would take was  a little unclear.</t>
+  </si>
+  <si>
+    <t>The researchers propose important work, but it presents more as a massive data curation project than an actual synthesis project. Shifting to a focus on what transformative science would come out of this effort would be more helpful and convincing. The likelihood of success in achieving this project (such as the development of the extraction pipeline and any difficulties in navigating the LLM portion of the textual data mining) is not fully explained.</t>
+  </si>
+  <si>
+    <t>There are an abundance of mass spectrometry-based proteomics data available in public repositories. The mining of these data, especially for the non-expert, are difficult for many reasons, including the lack of clearly associated metadata. The work outlined in the proposal is required in order to better use existing data sets to answer important questions in the molecular/cellular biosciences and to avoid redundant or unnecessary experiments. This section could have been strengthened by providing some clear examples of biological limitations due to the lack of metadata and some of the big picture questions that could be asked once the tools of the proposal are in place. 
+Significance: Making proteomics data and metadata more user-accessible to the non-expert is innovatitve and transformative. The working group also envisions that the machine learning tools developed here might also be used to explore other types of data sets.
+Rigor: The working group clearly describes the use of a test data set and a well-curated dataset to benchmark their workflows for identifying metadata. The working group also outlines steps to verify natural language processing algorithms are accurate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The working group has requested 2 years of NCEMS support and have a detailed timeline outlining milestones across those 2 years. Working as a team, and with NCEMS support, should allow the working group success in their aims. It would be helpful to see when in the timeline the working group plans to assemble or exchange personnel. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The proposal demonstrates a synthesis project, where publicly available proteomics data will be mined for the matching metadata. Tools will be designed to allow for the access to metadata by users of the proteomics repository. 
+The working group clearly identifies they will be working with mass spectrometry-based proteomics data in the PRIDE database, and outline specific data sets they are planning ot start with. They will also use open-access papers associated with the PRIDE datasets. PRIDE is the largest public repository of proteomics data, so the working group will have an abundance of data to build their model and tools. Limitations are minimal and acknowledged. 
+This portion could be improved by more clearly stating how the final data sets will be chosen. The group currently states that data sets will be "flexibily adjusted" during the group's activities.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The proposal is dedicated to making proteomics data findable, accessible, interoperable, and reusable. By pursuing the objectives outlined in the proposal, the group is clearly demonstrating a commitment to open and reproducible science principles. 
+The proposal also demonstrates an emphasis on team science, bringing together experts in bioinformatics, proteomics, and machine learning to accomplish their goals. The working group will also extend beyond those listed here through a community machine-learning challenge designed to develop the best open-source solutions for metadata access.
+The group also is comprised of three trainees. Their work on this project will allow for enhanced training of the next generation of data scientists. </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> The proposal addresses a key need in the proteomics community of making publically available data easier to mine and understand. There is an immense amount of data in the PRIDE and other proteomics repositories, but accessing the data and the experimental parameters (metadata) connected with these data can be daunting. It is necessary to develop tools to make proteomics data accessible to experts and non-experts alike. This will allow for new questions and observations in the molecular and cellular biosciences from existing datasets. This working group will help address this problem by developing tools that work with the PRIDE repository to extract metadata and make it clearly available with the raw proteomics data. The working group assembles experts from a range of fields to help solve this problem, and brings in a community machine-learning challenge to expand the reach and acquire new ideas. The proposal is clearly written, the timeline is aggressive but manageable, and the justification for NCEMS support is adequate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The proposal aims to address the critical challenge of metadata completeness and consistence in proteomics data, which is essential for understanding cellular mechanisms and disease processes. The integration of bioinformatics, NLP, and LLMs for automated metadata extraction represents a cutting-edge approach in the field. By enhancing metadata quality and usability, the proposal enables efficient data reuse, supports AI-driven analyses, and accelerates scientific discoveries in proteomics and related fields.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Overall, the goals and timelines are realistic. Extracting metadata from scientific manuscripts using NLP (Months 4–9) is a complex task, especially ensuring accuracy and avoiding hallucinations. This might require more time or iterative improvements. Allocating buffer time for this task would further enhance the likelihood of success.</t>
+  </si>
+  <si>
+    <t>The proposal clearly demonstrates a synthesis project and combines multiple disciplines and methodologies, including: Bioinformatics, Natural Language Processing (NLP), Machine Learning, Data Standards (SDRF-Proteomics format and controlled vocabularies), Software Development (integration into PRIDE and user-friendly tools like lesSDRF), with data sources clearly identified and the scope clearly defined.</t>
+  </si>
+  <si>
+    <t>The proposal clearly aligns with open, team-based, and reproducible scientific principles through its emphasis on open data and tools, interdisciplinary collaboration, community engagement, standardized workflows, and rigorous validation. These commitments ensure that the project's outcomes will be accessible, transparent, and reusable by the broader scientific community.</t>
+  </si>
+  <si>
+    <t>The proposal addresses the critical challenge of metadata completeness and consistency in proteomics data, essential for understanding cellular mechanisms and disease processes. Integrating bioinformatics, NLP, and LLMs for automated metadata extraction is an innovative approach that promises to enhance metadata quality and usability.
+To improve accuracy and avoid hallucinations, the proposal could benefit from iterative validation steps and feedback loops, involving multiple rounds of testing with expert input. Allocating additional buffer time for these tasks would help manage unforeseen challenges and ensure higher reliability.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -260,6 +1016,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -281,7 +1050,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -290,6 +1059,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -625,7 +1398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05BF02B-5287-7141-B8AA-133FE499772C}">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="6.1640625" customWidth="1"/>
@@ -858,6 +1631,1971 @@
         <v>3</v>
       </c>
     </row>
+    <row r="6" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="J6" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" t="s">
+        <v>41</v>
+      </c>
+      <c r="L6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="N6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J7" t="s">
+        <v>17</v>
+      </c>
+      <c r="K7" t="s">
+        <v>46</v>
+      </c>
+      <c r="L7" t="s">
+        <v>17</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="N7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="H8" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J8" t="s">
+        <v>17</v>
+      </c>
+      <c r="K8" t="s">
+        <v>51</v>
+      </c>
+      <c r="L8" t="s">
+        <v>17</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="N8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H9" t="s">
+        <v>17</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="J9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="L9" t="s">
+        <v>17</v>
+      </c>
+      <c r="M9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="N9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="404" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F10" t="s">
+        <v>17</v>
+      </c>
+      <c r="G10" t="s">
+        <v>60</v>
+      </c>
+      <c r="H10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="J10" t="s">
+        <v>17</v>
+      </c>
+      <c r="K10" t="s">
+        <v>62</v>
+      </c>
+      <c r="L10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M10" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="N10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="5">
+        <v>3</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="5">
+        <v>3</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="J11" t="s">
+        <v>17</v>
+      </c>
+      <c r="K11" t="s">
+        <v>67</v>
+      </c>
+      <c r="L11" t="s">
+        <v>17</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="N11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="5">
+        <v>3</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="5">
+        <v>4</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" t="s">
+        <v>70</v>
+      </c>
+      <c r="H12" t="s">
+        <v>17</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="J12" t="s">
+        <v>17</v>
+      </c>
+      <c r="K12" t="s">
+        <v>72</v>
+      </c>
+      <c r="L12" t="s">
+        <v>17</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="N12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13">
+        <v>4</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F13" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" t="s">
+        <v>76</v>
+      </c>
+      <c r="H13" t="s">
+        <v>17</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="J13" t="s">
+        <v>17</v>
+      </c>
+      <c r="K13" t="s">
+        <v>78</v>
+      </c>
+      <c r="L13" t="s">
+        <v>17</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="N13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14">
+        <v>4</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14">
+        <v>2</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F14" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" t="s">
+        <v>81</v>
+      </c>
+      <c r="H14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="J14" t="s">
+        <v>17</v>
+      </c>
+      <c r="K14" t="s">
+        <v>83</v>
+      </c>
+      <c r="L14" t="s">
+        <v>17</v>
+      </c>
+      <c r="M14" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="N14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15">
+        <v>4</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="F15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" t="s">
+        <v>86</v>
+      </c>
+      <c r="H15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J15" t="s">
+        <v>17</v>
+      </c>
+      <c r="K15" t="s">
+        <v>88</v>
+      </c>
+      <c r="L15" t="s">
+        <v>17</v>
+      </c>
+      <c r="M15" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="N15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16">
+        <v>4</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16">
+        <v>4</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="H16" t="s">
+        <v>17</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="J16" t="s">
+        <v>17</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="L16" t="s">
+        <v>17</v>
+      </c>
+      <c r="M16" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="N16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17">
+        <v>5</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F17" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" t="s">
+        <v>97</v>
+      </c>
+      <c r="H17" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="J17" t="s">
+        <v>17</v>
+      </c>
+      <c r="K17" t="s">
+        <v>99</v>
+      </c>
+      <c r="L17" t="s">
+        <v>17</v>
+      </c>
+      <c r="M17" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="N17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18">
+        <v>5</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="F18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="H18" t="s">
+        <v>17</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="J18" t="s">
+        <v>17</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="L18" t="s">
+        <v>17</v>
+      </c>
+      <c r="M18" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="N18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19">
+        <v>5</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D19">
+        <v>3</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F19" t="s">
+        <v>17</v>
+      </c>
+      <c r="G19" t="s">
+        <v>107</v>
+      </c>
+      <c r="H19" t="s">
+        <v>17</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="J19" t="s">
+        <v>17</v>
+      </c>
+      <c r="K19" t="s">
+        <v>109</v>
+      </c>
+      <c r="L19" t="s">
+        <v>17</v>
+      </c>
+      <c r="M19" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="N19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20">
+        <v>5</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D20">
+        <v>4</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="F20" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="H20" t="s">
+        <v>17</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="J20" t="s">
+        <v>17</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="L20" t="s">
+        <v>17</v>
+      </c>
+      <c r="M20" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="N20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21">
+        <v>6</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="F21" t="s">
+        <v>17</v>
+      </c>
+      <c r="G21" t="s">
+        <v>118</v>
+      </c>
+      <c r="H21" t="s">
+        <v>17</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="J21" t="s">
+        <v>17</v>
+      </c>
+      <c r="K21" t="s">
+        <v>120</v>
+      </c>
+      <c r="L21" t="s">
+        <v>17</v>
+      </c>
+      <c r="M21" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="N21" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22">
+        <v>6</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="F22" t="s">
+        <v>17</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="H22" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="J22" t="s">
+        <v>17</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="L22" t="s">
+        <v>17</v>
+      </c>
+      <c r="M22" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="N22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>1</v>
+      </c>
+      <c r="B23">
+        <v>6</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D23">
+        <v>3</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="F23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G23" t="s">
+        <v>128</v>
+      </c>
+      <c r="H23" t="s">
+        <v>17</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="J23" t="s">
+        <v>17</v>
+      </c>
+      <c r="K23" t="s">
+        <v>130</v>
+      </c>
+      <c r="L23" t="s">
+        <v>17</v>
+      </c>
+      <c r="M23" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="N23" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24">
+        <v>6</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D24">
+        <v>4</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="F24" t="s">
+        <v>17</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H24" t="s">
+        <v>17</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="J24" t="s">
+        <v>17</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="L24" t="s">
+        <v>17</v>
+      </c>
+      <c r="M24" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="N24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>1</v>
+      </c>
+      <c r="B25">
+        <v>7</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="F25">
+        <v>3</v>
+      </c>
+      <c r="G25" t="s">
+        <v>139</v>
+      </c>
+      <c r="H25">
+        <v>4</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="J25">
+        <v>5</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="L25">
+        <v>5</v>
+      </c>
+      <c r="M25" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="N25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="404" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26">
+        <v>7</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D26">
+        <v>2</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="F26">
+        <v>2</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="H26">
+        <v>2</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="J26">
+        <v>2</v>
+      </c>
+      <c r="K26" t="s">
+        <v>146</v>
+      </c>
+      <c r="L26">
+        <v>3</v>
+      </c>
+      <c r="M26" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="N26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27">
+        <v>7</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D27">
+        <v>3</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="F27" t="s">
+        <v>17</v>
+      </c>
+      <c r="G27" t="s">
+        <v>149</v>
+      </c>
+      <c r="H27" t="s">
+        <v>17</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="J27" t="s">
+        <v>17</v>
+      </c>
+      <c r="K27" t="s">
+        <v>151</v>
+      </c>
+      <c r="L27" t="s">
+        <v>17</v>
+      </c>
+      <c r="M27" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="N27" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>1</v>
+      </c>
+      <c r="B28">
+        <v>7</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D28">
+        <v>4</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F28" t="s">
+        <v>17</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="H28" t="s">
+        <v>17</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="J28" t="s">
+        <v>17</v>
+      </c>
+      <c r="K28" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="L28" t="s">
+        <v>17</v>
+      </c>
+      <c r="M28" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="N28" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>1</v>
+      </c>
+      <c r="B29">
+        <v>8</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D29">
+        <v>1</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="F29" t="s">
+        <v>17</v>
+      </c>
+      <c r="G29" t="s">
+        <v>160</v>
+      </c>
+      <c r="H29" t="s">
+        <v>17</v>
+      </c>
+      <c r="I29" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="J29" t="s">
+        <v>17</v>
+      </c>
+      <c r="K29" t="s">
+        <v>162</v>
+      </c>
+      <c r="L29" t="s">
+        <v>17</v>
+      </c>
+      <c r="M29" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="N29" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>1</v>
+      </c>
+      <c r="B30">
+        <v>8</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D30">
+        <v>2</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="F30" t="s">
+        <v>17</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="H30" t="s">
+        <v>17</v>
+      </c>
+      <c r="I30" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="J30" t="s">
+        <v>17</v>
+      </c>
+      <c r="K30" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="L30" t="s">
+        <v>17</v>
+      </c>
+      <c r="M30" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="N30" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>1</v>
+      </c>
+      <c r="B31">
+        <v>8</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D31">
+        <v>3</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="F31" t="s">
+        <v>17</v>
+      </c>
+      <c r="G31" t="s">
+        <v>170</v>
+      </c>
+      <c r="H31" t="s">
+        <v>17</v>
+      </c>
+      <c r="I31" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="J31" t="s">
+        <v>17</v>
+      </c>
+      <c r="K31" t="s">
+        <v>172</v>
+      </c>
+      <c r="L31" t="s">
+        <v>17</v>
+      </c>
+      <c r="M31" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="N31" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>1</v>
+      </c>
+      <c r="B32">
+        <v>8</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D32">
+        <v>4</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="F32" t="s">
+        <v>17</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="H32" t="s">
+        <v>17</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="J32" t="s">
+        <v>17</v>
+      </c>
+      <c r="K32" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="L32" t="s">
+        <v>17</v>
+      </c>
+      <c r="M32" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="N32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>1</v>
+      </c>
+      <c r="B33">
+        <v>8</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D33">
+        <v>5</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="F33" t="s">
+        <v>17</v>
+      </c>
+      <c r="G33" t="s">
+        <v>180</v>
+      </c>
+      <c r="H33" t="s">
+        <v>17</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="J33" t="s">
+        <v>17</v>
+      </c>
+      <c r="K33" t="s">
+        <v>182</v>
+      </c>
+      <c r="L33" t="s">
+        <v>17</v>
+      </c>
+      <c r="M33" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="N33" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>1</v>
+      </c>
+      <c r="B34">
+        <v>9</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="F34" t="s">
+        <v>17</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="H34" t="s">
+        <v>17</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="J34" t="s">
+        <v>17</v>
+      </c>
+      <c r="K34" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="L34" t="s">
+        <v>17</v>
+      </c>
+      <c r="M34" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="N34" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35">
+        <v>9</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D35">
+        <v>2</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F35" t="s">
+        <v>17</v>
+      </c>
+      <c r="G35" t="s">
+        <v>191</v>
+      </c>
+      <c r="H35" t="s">
+        <v>17</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="J35" t="s">
+        <v>17</v>
+      </c>
+      <c r="L35" t="s">
+        <v>17</v>
+      </c>
+      <c r="M35" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="N35" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>1</v>
+      </c>
+      <c r="B36">
+        <v>9</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D36">
+        <v>3</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F36" t="s">
+        <v>17</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="H36" t="s">
+        <v>17</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="J36" t="s">
+        <v>17</v>
+      </c>
+      <c r="K36" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="L36" t="s">
+        <v>17</v>
+      </c>
+      <c r="M36" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="N36" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>1</v>
+      </c>
+      <c r="B37">
+        <v>10</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="D37">
+        <v>1</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="F37">
+        <v>4.3</v>
+      </c>
+      <c r="G37" t="s">
+        <v>201</v>
+      </c>
+      <c r="H37" t="s">
+        <v>17</v>
+      </c>
+      <c r="I37" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="J37" t="s">
+        <v>17</v>
+      </c>
+      <c r="K37" t="s">
+        <v>203</v>
+      </c>
+      <c r="L37" t="s">
+        <v>17</v>
+      </c>
+      <c r="M37" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="N37" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>1</v>
+      </c>
+      <c r="B38">
+        <v>10</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="D38">
+        <v>2</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="F38" t="s">
+        <v>17</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="H38" t="s">
+        <v>17</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="J38" t="s">
+        <v>17</v>
+      </c>
+      <c r="K38" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="L38" t="s">
+        <v>17</v>
+      </c>
+      <c r="M38" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="N38" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>1</v>
+      </c>
+      <c r="B39">
+        <v>10</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="D39">
+        <v>3</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="F39" t="s">
+        <v>17</v>
+      </c>
+      <c r="G39" t="s">
+        <v>211</v>
+      </c>
+      <c r="H39" t="s">
+        <v>17</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="J39" t="s">
+        <v>17</v>
+      </c>
+      <c r="K39" t="s">
+        <v>213</v>
+      </c>
+      <c r="L39" t="s">
+        <v>17</v>
+      </c>
+      <c r="M39" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="N39" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>1</v>
+      </c>
+      <c r="B40">
+        <v>10</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="D40">
+        <v>4</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="F40" t="s">
+        <v>17</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="H40" t="s">
+        <v>17</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="J40" t="s">
+        <v>17</v>
+      </c>
+      <c r="K40" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="L40" t="s">
+        <v>17</v>
+      </c>
+      <c r="M40" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="N40" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>1</v>
+      </c>
+      <c r="B41">
+        <v>11</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="D41">
+        <v>1</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="F41">
+        <v>4</v>
+      </c>
+      <c r="G41" t="s">
+        <v>222</v>
+      </c>
+      <c r="H41">
+        <v>4</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J41">
+        <v>3</v>
+      </c>
+      <c r="K41" t="s">
+        <v>224</v>
+      </c>
+      <c r="L41">
+        <v>5</v>
+      </c>
+      <c r="M41" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="N41">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>1</v>
+      </c>
+      <c r="B42">
+        <v>11</v>
+      </c>
+      <c r="D42">
+        <v>2</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="F42" t="s">
+        <v>17</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="H42" t="s">
+        <v>17</v>
+      </c>
+      <c r="I42" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="J42" t="s">
+        <v>17</v>
+      </c>
+      <c r="K42" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="L42" t="s">
+        <v>17</v>
+      </c>
+      <c r="M42" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="N42" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>1</v>
+      </c>
+      <c r="B43">
+        <v>11</v>
+      </c>
+      <c r="D43">
+        <v>3</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="F43" t="s">
+        <v>17</v>
+      </c>
+      <c r="G43" t="s">
+        <v>232</v>
+      </c>
+      <c r="H43" t="s">
+        <v>17</v>
+      </c>
+      <c r="I43" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="J43" t="s">
+        <v>17</v>
+      </c>
+      <c r="K43" t="s">
+        <v>234</v>
+      </c>
+      <c r="L43" t="s">
+        <v>17</v>
+      </c>
+      <c r="M43" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="N43" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>1</v>
+      </c>
+      <c r="B44">
+        <v>11</v>
+      </c>
+      <c r="D44">
+        <v>4</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F44" t="s">
+        <v>17</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="H44" t="s">
+        <v>17</v>
+      </c>
+      <c r="I44" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="J44" t="s">
+        <v>17</v>
+      </c>
+      <c r="K44" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="L44" t="s">
+        <v>17</v>
+      </c>
+      <c r="M44" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="N44" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" ht="340" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>1</v>
+      </c>
+      <c r="B45">
+        <v>12</v>
+      </c>
+      <c r="C45" t="s">
+        <v>241</v>
+      </c>
+      <c r="D45">
+        <v>1</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="F45" t="s">
+        <v>17</v>
+      </c>
+      <c r="G45" t="s">
+        <v>243</v>
+      </c>
+      <c r="H45" t="s">
+        <v>17</v>
+      </c>
+      <c r="I45" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="J45" t="s">
+        <v>17</v>
+      </c>
+      <c r="K45" t="s">
+        <v>245</v>
+      </c>
+      <c r="L45" t="s">
+        <v>17</v>
+      </c>
+      <c r="M45" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="N45" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>1</v>
+      </c>
+      <c r="B46">
+        <v>12</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="D46">
+        <v>2</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="F46" t="s">
+        <v>17</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="H46" t="s">
+        <v>17</v>
+      </c>
+      <c r="I46" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="J46" t="s">
+        <v>17</v>
+      </c>
+      <c r="K46" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="L46" t="s">
+        <v>17</v>
+      </c>
+      <c r="M46" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="N46" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>1</v>
+      </c>
+      <c r="B47">
+        <v>12</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="D47">
+        <v>3</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="F47" t="s">
+        <v>17</v>
+      </c>
+      <c r="G47" t="s">
+        <v>253</v>
+      </c>
+      <c r="H47" t="s">
+        <v>17</v>
+      </c>
+      <c r="I47" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="J47" t="s">
+        <v>17</v>
+      </c>
+      <c r="K47" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="L47" t="s">
+        <v>17</v>
+      </c>
+      <c r="M47" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="N47" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>1</v>
+      </c>
+      <c r="B48">
+        <v>12</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="D48">
+        <v>4</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="F48" t="s">
+        <v>17</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="H48" t="s">
+        <v>17</v>
+      </c>
+      <c r="I48" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="J48" t="s">
+        <v>17</v>
+      </c>
+      <c r="K48" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="L48" t="s">
+        <v>17</v>
+      </c>
+      <c r="M48" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="N48" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>